<commit_message>
upload: crew_stats for 2025-11-05 (051125/Crewstats.xlsx)
</commit_message>
<xml_diff>
--- a/outputs/2025-11-05/inputs/crew_stats.xlsx
+++ b/outputs/2025-11-05/inputs/crew_stats.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29929"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\Crew Sched and BD Shared Folder\2025\November\Processed data\051125\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\Flight Operations\Crew Sched and BD Shared Folder\2025\November\Input Files\KTree\051125\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59623806-0D5C-4DAD-AB6C-A9654C4FA121}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38280" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="2025-11-05" sheetId="1" r:id="rId1"/>
@@ -3655,18 +3655,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M235"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="18" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="19" bestFit="1" customWidth="1"/>
-    <col min="7" max="13" width="3.85546875" bestFit="1" customWidth="1"/>
+    <col min="7" max="13" width="3.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1088</v>
       </c>
@@ -3707,7 +3707,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -3736,7 +3736,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -3768,7 +3768,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -3800,7 +3800,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>15</v>
       </c>
@@ -3832,7 +3832,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>16</v>
       </c>
@@ -3846,7 +3846,7 @@
         <v>1008</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>17</v>
       </c>
@@ -3860,7 +3860,7 @@
         <v>1009</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -3892,7 +3892,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>19</v>
       </c>
@@ -3924,7 +3924,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>20</v>
       </c>
@@ -3956,7 +3956,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>21</v>
       </c>
@@ -3979,7 +3979,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>22</v>
       </c>
@@ -4011,7 +4011,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>23</v>
       </c>
@@ -4043,7 +4043,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>24</v>
       </c>
@@ -4072,7 +4072,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>25</v>
       </c>
@@ -4104,7 +4104,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>26</v>
       </c>
@@ -4136,7 +4136,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="17" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>27</v>
       </c>
@@ -4165,7 +4165,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="18" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>28</v>
       </c>
@@ -4197,7 +4197,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="19" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>29</v>
       </c>
@@ -4226,7 +4226,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="20" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>30</v>
       </c>
@@ -4252,7 +4252,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -4284,7 +4284,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="22" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>32</v>
       </c>
@@ -4313,7 +4313,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="23" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>33</v>
       </c>
@@ -4345,7 +4345,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="24" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>34</v>
       </c>
@@ -4377,7 +4377,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="25" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>35</v>
       </c>
@@ -4406,7 +4406,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>36</v>
       </c>
@@ -4438,7 +4438,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="27" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>37</v>
       </c>
@@ -4470,7 +4470,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>38</v>
       </c>
@@ -4502,7 +4502,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>39</v>
       </c>
@@ -4531,7 +4531,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="30" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>40</v>
       </c>
@@ -4563,7 +4563,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="31" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>41</v>
       </c>
@@ -4595,7 +4595,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="32" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>42</v>
       </c>
@@ -4624,7 +4624,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="33" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>43</v>
       </c>
@@ -4638,7 +4638,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="34" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>44</v>
       </c>
@@ -4658,7 +4658,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="35" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>45</v>
       </c>
@@ -4675,7 +4675,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="36" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>46</v>
       </c>
@@ -4701,7 +4701,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="37" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>47</v>
       </c>
@@ -4727,7 +4727,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="38" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>48</v>
       </c>
@@ -4756,7 +4756,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="39" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>49</v>
       </c>
@@ -4788,7 +4788,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="40" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>50</v>
       </c>
@@ -4817,7 +4817,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="41" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>51</v>
       </c>
@@ -4849,7 +4849,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="42" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>52</v>
       </c>
@@ -4878,7 +4878,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="43" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>53</v>
       </c>
@@ -4886,7 +4886,7 @@
         <v>508</v>
       </c>
     </row>
-    <row r="44" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>54</v>
       </c>
@@ -4915,7 +4915,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="45" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>55</v>
       </c>
@@ -4947,7 +4947,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="46" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>56</v>
       </c>
@@ -4979,7 +4979,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>57</v>
       </c>
@@ -5011,7 +5011,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="48" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>58</v>
       </c>
@@ -5031,7 +5031,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="49" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>59</v>
       </c>
@@ -5048,7 +5048,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="50" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>60</v>
       </c>
@@ -5077,7 +5077,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>61</v>
       </c>
@@ -5109,7 +5109,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="52" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>62</v>
       </c>
@@ -5138,7 +5138,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="53" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>63</v>
       </c>
@@ -5161,7 +5161,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="54" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>64</v>
       </c>
@@ -5175,7 +5175,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="55" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>65</v>
       </c>
@@ -5207,7 +5207,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="56" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>66</v>
       </c>
@@ -5239,7 +5239,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="57" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>67</v>
       </c>
@@ -5259,7 +5259,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="58" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>68</v>
       </c>
@@ -5288,7 +5288,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="59" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>69</v>
       </c>
@@ -5317,7 +5317,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="60" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>70</v>
       </c>
@@ -5349,7 +5349,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="61" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>71</v>
       </c>
@@ -5363,7 +5363,7 @@
         <v>747</v>
       </c>
     </row>
-    <row r="62" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>72</v>
       </c>
@@ -5383,7 +5383,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="63" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>73</v>
       </c>
@@ -5412,7 +5412,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="64" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>74</v>
       </c>
@@ -5432,7 +5432,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="65" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>75</v>
       </c>
@@ -5464,7 +5464,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="66" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>76</v>
       </c>
@@ -5493,7 +5493,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="67" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>77</v>
       </c>
@@ -5522,7 +5522,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="68" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>78</v>
       </c>
@@ -5551,7 +5551,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="69" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>79</v>
       </c>
@@ -5583,7 +5583,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="70" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>80</v>
       </c>
@@ -5612,7 +5612,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="71" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>81</v>
       </c>
@@ -5638,7 +5638,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="72" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>82</v>
       </c>
@@ -5670,7 +5670,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="73" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>83</v>
       </c>
@@ -5696,7 +5696,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="74" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>84</v>
       </c>
@@ -5728,7 +5728,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="75" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>85</v>
       </c>
@@ -5757,7 +5757,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="76" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>86</v>
       </c>
@@ -5786,7 +5786,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="77" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>87</v>
       </c>
@@ -5806,7 +5806,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="78" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>88</v>
       </c>
@@ -5838,7 +5838,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="79" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>89</v>
       </c>
@@ -5867,7 +5867,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="80" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>90</v>
       </c>
@@ -5899,7 +5899,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>91</v>
       </c>
@@ -5931,7 +5931,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="82" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>92</v>
       </c>
@@ -5963,7 +5963,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="83" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>93</v>
       </c>
@@ -5995,7 +5995,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="84" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>94</v>
       </c>
@@ -6024,7 +6024,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="85" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>95</v>
       </c>
@@ -6053,7 +6053,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="86" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>96</v>
       </c>
@@ -6085,7 +6085,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="87" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>97</v>
       </c>
@@ -6114,7 +6114,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="88" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>98</v>
       </c>
@@ -6140,7 +6140,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="89" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>99</v>
       </c>
@@ -6172,7 +6172,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="90" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>100</v>
       </c>
@@ -6201,7 +6201,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="91" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>101</v>
       </c>
@@ -6230,7 +6230,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="92" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>102</v>
       </c>
@@ -6259,7 +6259,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="93" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>103</v>
       </c>
@@ -6288,7 +6288,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="94" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>104</v>
       </c>
@@ -6320,7 +6320,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="95" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>105</v>
       </c>
@@ -6340,7 +6340,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="96" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>106</v>
       </c>
@@ -6372,7 +6372,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="97" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>107</v>
       </c>
@@ -6401,7 +6401,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="98" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>108</v>
       </c>
@@ -6433,7 +6433,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="99" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>109</v>
       </c>
@@ -6465,7 +6465,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="100" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>110</v>
       </c>
@@ -6491,7 +6491,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="101" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>111</v>
       </c>
@@ -6523,7 +6523,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>112</v>
       </c>
@@ -6552,7 +6552,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="103" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>113</v>
       </c>
@@ -6584,7 +6584,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="104" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>114</v>
       </c>
@@ -6613,7 +6613,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="105" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>115</v>
       </c>
@@ -6645,7 +6645,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="106" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>116</v>
       </c>
@@ -6674,7 +6674,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="107" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>117</v>
       </c>
@@ -6706,7 +6706,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="108" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>118</v>
       </c>
@@ -6738,7 +6738,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="109" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>119</v>
       </c>
@@ -6764,7 +6764,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="110" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>120</v>
       </c>
@@ -6790,7 +6790,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="111" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>121</v>
       </c>
@@ -6816,7 +6816,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="112" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>122</v>
       </c>
@@ -6848,7 +6848,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="113" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>123</v>
       </c>
@@ -6874,7 +6874,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="114" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>124</v>
       </c>
@@ -6906,7 +6906,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="115" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>125</v>
       </c>
@@ -6932,7 +6932,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="116" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>126</v>
       </c>
@@ -6961,7 +6961,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="117" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>127</v>
       </c>
@@ -6990,7 +6990,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="118" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>128</v>
       </c>
@@ -7022,7 +7022,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="119" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>129</v>
       </c>
@@ -7048,7 +7048,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="120" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>130</v>
       </c>
@@ -7080,7 +7080,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="121" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>131</v>
       </c>
@@ -7106,7 +7106,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="122" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A122" t="s">
         <v>132</v>
       </c>
@@ -7138,7 +7138,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="123" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A123" t="s">
         <v>133</v>
       </c>
@@ -7167,7 +7167,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="124" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A124" t="s">
         <v>134</v>
       </c>
@@ -7193,7 +7193,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="125" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A125" t="s">
         <v>135</v>
       </c>
@@ -7222,7 +7222,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="126" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A126" t="s">
         <v>136</v>
       </c>
@@ -7254,7 +7254,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="127" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A127" t="s">
         <v>137</v>
       </c>
@@ -7286,7 +7286,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="128" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A128" t="s">
         <v>138</v>
       </c>
@@ -7306,7 +7306,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="129" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A129" t="s">
         <v>139</v>
       </c>
@@ -7338,7 +7338,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="130" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A130" t="s">
         <v>140</v>
       </c>
@@ -7370,7 +7370,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="131" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A131" t="s">
         <v>141</v>
       </c>
@@ -7399,7 +7399,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="132" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A132" t="s">
         <v>142</v>
       </c>
@@ -7428,7 +7428,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="133" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A133" t="s">
         <v>143</v>
       </c>
@@ -7457,7 +7457,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="134" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A134" t="s">
         <v>144</v>
       </c>
@@ -7489,7 +7489,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="135" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A135" t="s">
         <v>145</v>
       </c>
@@ -7521,7 +7521,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="136" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A136" t="s">
         <v>146</v>
       </c>
@@ -7553,7 +7553,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="137" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A137" t="s">
         <v>147</v>
       </c>
@@ -7579,7 +7579,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="138" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A138" t="s">
         <v>148</v>
       </c>
@@ -7611,7 +7611,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="139" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A139" t="s">
         <v>149</v>
       </c>
@@ -7637,7 +7637,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="140" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A140" t="s">
         <v>150</v>
       </c>
@@ -7657,7 +7657,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="141" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A141" t="s">
         <v>151</v>
       </c>
@@ -7689,7 +7689,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="142" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A142" t="s">
         <v>152</v>
       </c>
@@ -7721,7 +7721,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="143" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A143" t="s">
         <v>153</v>
       </c>
@@ -7747,7 +7747,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="144" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A144" t="s">
         <v>154</v>
       </c>
@@ -7779,7 +7779,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="145" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A145" t="s">
         <v>155</v>
       </c>
@@ -7802,7 +7802,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="146" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A146" t="s">
         <v>156</v>
       </c>
@@ -7831,7 +7831,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="147" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A147" t="s">
         <v>157</v>
       </c>
@@ -7863,7 +7863,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="148" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A148" t="s">
         <v>158</v>
       </c>
@@ -7892,7 +7892,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="149" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A149" t="s">
         <v>159</v>
       </c>
@@ -7921,7 +7921,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="150" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A150" t="s">
         <v>160</v>
       </c>
@@ -7953,7 +7953,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="151" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A151" t="s">
         <v>161</v>
       </c>
@@ -7985,7 +7985,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="152" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A152" t="s">
         <v>162</v>
       </c>
@@ -8014,7 +8014,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="153" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A153" t="s">
         <v>163</v>
       </c>
@@ -8046,7 +8046,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="154" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A154" t="s">
         <v>164</v>
       </c>
@@ -8075,7 +8075,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="155" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A155" t="s">
         <v>165</v>
       </c>
@@ -8101,7 +8101,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="156" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A156" t="s">
         <v>166</v>
       </c>
@@ -8133,7 +8133,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="157" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A157" t="s">
         <v>167</v>
       </c>
@@ -8162,7 +8162,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="158" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A158" t="s">
         <v>168</v>
       </c>
@@ -8194,7 +8194,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="159" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A159" t="s">
         <v>169</v>
       </c>
@@ -8214,7 +8214,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="160" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A160" t="s">
         <v>170</v>
       </c>
@@ -8240,7 +8240,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="161" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A161" t="s">
         <v>171</v>
       </c>
@@ -8272,7 +8272,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="162" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A162" t="s">
         <v>172</v>
       </c>
@@ -8301,7 +8301,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="163" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A163" t="s">
         <v>173</v>
       </c>
@@ -8327,7 +8327,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="164" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A164" t="s">
         <v>174</v>
       </c>
@@ -8359,7 +8359,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="165" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A165" t="s">
         <v>175</v>
       </c>
@@ -8391,7 +8391,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="166" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A166" t="s">
         <v>176</v>
       </c>
@@ -8423,7 +8423,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="167" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A167" t="s">
         <v>177</v>
       </c>
@@ -8455,7 +8455,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="168" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A168" t="s">
         <v>178</v>
       </c>
@@ -8469,7 +8469,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="169" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A169" t="s">
         <v>179</v>
       </c>
@@ -8498,7 +8498,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="170" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A170" t="s">
         <v>180</v>
       </c>
@@ -8530,7 +8530,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="171" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A171" t="s">
         <v>181</v>
       </c>
@@ -8562,7 +8562,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="172" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A172" t="s">
         <v>182</v>
       </c>
@@ -8594,7 +8594,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="173" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A173" t="s">
         <v>183</v>
       </c>
@@ -8626,7 +8626,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="174" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A174" t="s">
         <v>184</v>
       </c>
@@ -8655,7 +8655,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="175" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A175" t="s">
         <v>185</v>
       </c>
@@ -8687,7 +8687,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="176" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A176" t="s">
         <v>186</v>
       </c>
@@ -8719,7 +8719,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="177" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A177" t="s">
         <v>187</v>
       </c>
@@ -8751,7 +8751,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="178" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A178" t="s">
         <v>188</v>
       </c>
@@ -8783,7 +8783,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="179" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A179" t="s">
         <v>189</v>
       </c>
@@ -8803,7 +8803,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="180" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A180" t="s">
         <v>190</v>
       </c>
@@ -8835,7 +8835,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="181" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A181" t="s">
         <v>191</v>
       </c>
@@ -8858,7 +8858,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="182" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A182" t="s">
         <v>192</v>
       </c>
@@ -8890,7 +8890,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="183" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A183" t="s">
         <v>193</v>
       </c>
@@ -8919,7 +8919,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="184" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A184" t="s">
         <v>194</v>
       </c>
@@ -8945,7 +8945,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="185" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A185" t="s">
         <v>195</v>
       </c>
@@ -8977,7 +8977,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="186" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A186" t="s">
         <v>196</v>
       </c>
@@ -8997,7 +8997,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="187" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A187" t="s">
         <v>197</v>
       </c>
@@ -9029,7 +9029,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="188" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A188" t="s">
         <v>198</v>
       </c>
@@ -9058,7 +9058,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="189" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A189" t="s">
         <v>199</v>
       </c>
@@ -9090,7 +9090,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="190" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A190" t="s">
         <v>200</v>
       </c>
@@ -9119,7 +9119,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="191" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A191" t="s">
         <v>201</v>
       </c>
@@ -9148,7 +9148,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="192" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A192" t="s">
         <v>202</v>
       </c>
@@ -9177,7 +9177,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="193" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A193" t="s">
         <v>203</v>
       </c>
@@ -9203,7 +9203,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="194" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A194" t="s">
         <v>204</v>
       </c>
@@ -9235,7 +9235,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="195" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A195" t="s">
         <v>205</v>
       </c>
@@ -9264,7 +9264,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="196" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A196" t="s">
         <v>206</v>
       </c>
@@ -9293,7 +9293,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="197" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A197" t="s">
         <v>207</v>
       </c>
@@ -9322,7 +9322,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="198" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A198" t="s">
         <v>208</v>
       </c>
@@ -9354,7 +9354,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="199" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A199" t="s">
         <v>209</v>
       </c>
@@ -9374,7 +9374,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="200" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A200" t="s">
         <v>210</v>
       </c>
@@ -9403,7 +9403,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="201" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A201" t="s">
         <v>211</v>
       </c>
@@ -9435,7 +9435,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="202" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A202" t="s">
         <v>212</v>
       </c>
@@ -9467,7 +9467,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="203" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A203" t="s">
         <v>213</v>
       </c>
@@ -9499,7 +9499,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="204" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A204" t="s">
         <v>214</v>
       </c>
@@ -9531,7 +9531,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="205" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A205" t="s">
         <v>215</v>
       </c>
@@ -9554,7 +9554,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="206" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A206" t="s">
         <v>216</v>
       </c>
@@ -9583,7 +9583,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="207" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A207" t="s">
         <v>217</v>
       </c>
@@ -9615,7 +9615,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="208" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A208" t="s">
         <v>218</v>
       </c>
@@ -9647,7 +9647,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="209" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A209" t="s">
         <v>219</v>
       </c>
@@ -9679,7 +9679,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="210" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A210" t="s">
         <v>220</v>
       </c>
@@ -9699,7 +9699,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="211" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A211" t="s">
         <v>221</v>
       </c>
@@ -9731,7 +9731,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="212" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A212" t="s">
         <v>222</v>
       </c>
@@ -9757,7 +9757,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="213" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A213" t="s">
         <v>223</v>
       </c>
@@ -9786,7 +9786,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="214" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A214" t="s">
         <v>224</v>
       </c>
@@ -9797,7 +9797,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="215" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A215" t="s">
         <v>225</v>
       </c>
@@ -9826,7 +9826,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="216" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A216" t="s">
         <v>226</v>
       </c>
@@ -9858,7 +9858,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="217" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A217" t="s">
         <v>227</v>
       </c>
@@ -9890,7 +9890,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="218" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A218" t="s">
         <v>228</v>
       </c>
@@ -9919,7 +9919,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="219" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A219" t="s">
         <v>229</v>
       </c>
@@ -9948,7 +9948,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="220" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A220" t="s">
         <v>230</v>
       </c>
@@ -9974,7 +9974,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="221" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A221" t="s">
         <v>231</v>
       </c>
@@ -10006,7 +10006,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="222" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A222" t="s">
         <v>232</v>
       </c>
@@ -10038,7 +10038,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="223" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A223" t="s">
         <v>233</v>
       </c>
@@ -10070,7 +10070,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="224" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A224" t="s">
         <v>234</v>
       </c>
@@ -10096,7 +10096,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="225" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A225" t="s">
         <v>235</v>
       </c>
@@ -10128,7 +10128,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="226" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A226" t="s">
         <v>236</v>
       </c>
@@ -10157,7 +10157,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="227" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A227" t="s">
         <v>237</v>
       </c>
@@ -10186,7 +10186,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="228" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A228" t="s">
         <v>238</v>
       </c>
@@ -10206,7 +10206,7 @@
         <v>1015</v>
       </c>
     </row>
-    <row r="229" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A229" t="s">
         <v>239</v>
       </c>
@@ -10238,7 +10238,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="230" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A230" t="s">
         <v>240</v>
       </c>
@@ -10267,7 +10267,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="231" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A231" t="s">
         <v>241</v>
       </c>
@@ -10296,7 +10296,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="232" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A232" t="s">
         <v>242</v>
       </c>
@@ -10322,7 +10322,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="233" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A233" t="s">
         <v>243</v>
       </c>
@@ -10354,7 +10354,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="234" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A234" t="s">
         <v>244</v>
       </c>
@@ -10383,7 +10383,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="235" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:13" x14ac:dyDescent="0.3">
       <c r="A235" t="s">
         <v>245</v>
       </c>

</xml_diff>